<commit_message>
PETME2: final draft after all-agent review - per-target low-end bids, Brand campaign, paused out-of-stock groups
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HHS1qB7cDk7kf96VcdcLix
</commit_message>
<xml_diff>
--- a/petme2-ads-agent/outbox/2026-10-04/bulk-upload-2-new-campaigns.xlsx
+++ b/petme2-ads-agent/outbox/2026-10-04/bulk-upload-2-new-campaigns.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y82"/>
+  <dimension ref="A1:Y84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4">
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -936,7 +936,7 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
@@ -976,7 +976,7 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="14">
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="S15" t="n">
-        <v>0.55</v>
+        <v>0.65</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="S16" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="S18" t="n">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="S19" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
@@ -1293,7 +1293,7 @@
         </is>
       </c>
       <c r="S20" t="n">
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="22">
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="S23" t="n">
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="S26" t="n">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="S27" t="n">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="S28" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Competitors - Fountains</t>
+          <t>Competitors - $19.99 Fountains</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="R29" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="30">
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="S36" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="S37" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
         </is>
       </c>
       <c r="S38" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V39" t="inlineStr">
         <is>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ad Group</t>
+          <t>Campaign Negative Keyword</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2080,23 +2080,20 @@
           <t>PETME2-SP-AllProducts</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>More-Fountains22</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>2.2L Fountains - Exact</t>
-        </is>
-      </c>
       <c r="O40" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="R40" t="n">
-        <v>0.3</v>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>petme2</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>negativePhrase</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -2107,7 +2104,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Ad Group</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2125,15 +2122,18 @@
           <t>More-Fountains22</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>2.2L Fountains - Exact (AllProd)</t>
+        </is>
+      </c>
       <c r="O41" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>SD-85ET-IOZ3</t>
-        </is>
+      <c r="R41" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="42">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>JE-LQEW-9EHL</t>
+          <t>SD-85ET-IOZ3</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Keyword</t>
+          <t>Product Ad</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2204,17 +2204,9 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="S43" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>2.2l cat water fountain</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>exact</t>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>JE-LQEW-9EHL</t>
         </is>
       </c>
     </row>
@@ -2250,11 +2242,11 @@
         </is>
       </c>
       <c r="S44" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>cat water fountain with filter</t>
+          <t>automatic cat water fountain</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2295,11 +2287,11 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>small cat water fountain</t>
+          <t>cat water fountain with filter</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
@@ -2344,7 +2336,7 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>automatic cat water fountain</t>
+          <t>small cat water fountain</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
@@ -2389,7 +2381,7 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>74oz cat water fountain</t>
+          <t>2.2l cat water fountain</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -2406,7 +2398,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ad Group</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2421,12 +2413,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>More-Brand</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>PETME2 Brand - Exact</t>
+          <t>More-Fountains22</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -2434,8 +2421,18 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="R48" t="n">
-        <v>0.3</v>
+      <c r="S48" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>74oz cat water fountain</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -2446,7 +2443,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Ad Group</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2461,18 +2458,21 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Grooming</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Grooming - Exact (OUT OF STOCK - paused)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>QO-7VBS-CVT4</t>
-        </is>
+          <t>paused</t>
+        </is>
+      </c>
+      <c r="R49" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="50">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Grooming</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>LW-EZAJ-KKZD</t>
+          <t>GROOMING_KIT</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Grooming</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>93-E8EG-20UY</t>
+          <t>GROOMING_VACUUM</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Grooming</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>2H-2T1T-CJC3</t>
+          <t>MULTI_GROOMNG_KIT</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Grooming</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -2617,9 +2617,17 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>QY-HHE8-0H1B</t>
+      <c r="S53" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>dog grooming vacuum</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>exact</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2639,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2646,7 +2654,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Grooming</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -2654,9 +2662,17 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="Q54" t="inlineStr">
-        <is>
-          <t>L6-L3S1-I7Q6</t>
+      <c r="S54" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>pet grooming vacuum</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>exact</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2684,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Ad Group</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2683,18 +2699,21 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Supplement</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Supplement - Exact (OUT OF STOCK - paused)</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>SD-85ET-IOZ3</t>
-        </is>
+          <t>paused</t>
+        </is>
+      </c>
+      <c r="R55" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="56">
@@ -2720,7 +2739,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Supplement</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -2730,7 +2749,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>JE-LQEW-9EHL</t>
+          <t>Cat-Skin-&amp;-Coat-Supplement</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2776,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Supplement</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -2766,11 +2785,11 @@
         </is>
       </c>
       <c r="S57" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>petme2</t>
+          <t>cat skin and coat supplement</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
@@ -2802,7 +2821,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Supplement</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
@@ -2815,7 +2834,7 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>petme2 cat feeder</t>
+          <t>cat vitamins for skin and coat</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
@@ -2847,7 +2866,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>More-Brand</t>
+          <t>More-Supplement</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -2860,7 +2879,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>petme2 cat water fountain</t>
+          <t>cat shedding supplement</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
@@ -2892,21 +2911,21 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>More-Filters</t>
+          <t>More-FeederWaterer</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Filters - Exact (out of stock)</t>
+          <t>Feeder + Waterer - Exact (OUT OF STOCK - paused)</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="R60" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="61">
@@ -2932,7 +2951,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>More-Filters</t>
+          <t>More-FeederWaterer</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -2942,7 +2961,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>2L-Filter</t>
+          <t>2in1_FEEDER</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2988,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>More-Filters</t>
+          <t>More-FeederWaterer</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -2979,7 +2998,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>2.2Ltr-Filter-Transparent</t>
+          <t>FEEDER_X_WATERER</t>
         </is>
       </c>
     </row>
@@ -2991,7 +3010,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3006,7 +3025,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>More-Filters</t>
+          <t>More-FeederWaterer</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -3014,9 +3033,17 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
-        <is>
-          <t>2.2L-Filter</t>
+      <c r="S63" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>automatic cat feeder and water dispenser</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>exact</t>
         </is>
       </c>
     </row>
@@ -3028,7 +3055,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Campaign</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3038,22 +3065,35 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>More-Filters</t>
+          <t>PETME2-SP-Brand</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>PETME2 | SP | Brand | Exact</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>20261004</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Manual</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="Q64" t="inlineStr">
-        <is>
-          <t>3.2L-Stainless-Steel-Filter</t>
+          <t>paused</t>
+        </is>
+      </c>
+      <c r="P64" t="n">
+        <v>3</v>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>Dynamic bids - down only</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3105,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Ad Group</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3075,12 +3115,17 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>More-Filters</t>
+          <t>Brand-All</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>PETME2 Brand - Exact</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -3088,10 +3133,8 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="Q65" t="inlineStr">
-        <is>
-          <t>2.2Litre-Filter-Transparent</t>
-        </is>
+      <c r="R65" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="66">
@@ -3102,7 +3145,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Keyword</t>
+          <t>Product Ad</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3112,12 +3155,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>More-Filters</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -3125,17 +3168,9 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="S66" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T66" t="inlineStr">
-        <is>
-          <t>petme2 filter</t>
-        </is>
-      </c>
-      <c r="U66" t="inlineStr">
-        <is>
-          <t>exact</t>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>QO-7VBS-CVT4</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3182,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Keyword</t>
+          <t>Product Ad</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3157,12 +3192,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>More-Filters</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -3170,17 +3205,9 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="S67" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T67" t="inlineStr">
-        <is>
-          <t>petme2 fountain filter</t>
-        </is>
-      </c>
-      <c r="U67" t="inlineStr">
-        <is>
-          <t>exact</t>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>LW-EZAJ-KKZD</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3219,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Ad Group</t>
+          <t>Product Ad</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3202,17 +3229,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>More-Grooming</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>Grooming - Exact (out of stock)</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -3220,8 +3242,10 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="R68" t="n">
-        <v>0.4</v>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>93-E8EG-20UY</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -3242,12 +3266,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>More-Grooming</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -3257,7 +3281,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>GROOMING_KIT</t>
+          <t>2H-2T1T-CJC3</t>
         </is>
       </c>
     </row>
@@ -3279,12 +3303,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>More-Grooming</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -3294,7 +3318,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>GROOMING_VACUUM</t>
+          <t>QY-HHE8-0H1B</t>
         </is>
       </c>
     </row>
@@ -3316,12 +3340,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>More-Grooming</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -3331,7 +3355,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>MULTI_GROOMNG_KIT</t>
+          <t>L6-L3S1-I7Q6</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3367,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Keyword</t>
+          <t>Product Ad</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3353,12 +3377,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>More-Grooming</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -3366,17 +3390,9 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="S72" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>dog grooming vacuum</t>
-        </is>
-      </c>
-      <c r="U72" t="inlineStr">
-        <is>
-          <t>exact</t>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>SD-85ET-IOZ3</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3404,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Keyword</t>
+          <t>Product Ad</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3398,12 +3414,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>More-Grooming</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -3411,17 +3427,9 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="S73" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="T73" t="inlineStr">
-        <is>
-          <t>pet grooming vacuum</t>
-        </is>
-      </c>
-      <c r="U73" t="inlineStr">
-        <is>
-          <t>exact</t>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>JE-LQEW-9EHL</t>
         </is>
       </c>
     </row>
@@ -3433,7 +3441,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ad Group</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3443,17 +3451,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>More-Supplement</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>Supplement - Exact (out of stock)</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -3461,8 +3464,18 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="R74" t="n">
-        <v>0.3</v>
+      <c r="S74" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>petme2</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -3473,7 +3486,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Product Ad</t>
+          <t>Keyword</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3483,12 +3496,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>More-Supplement</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -3496,9 +3509,17 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="Q75" t="inlineStr">
-        <is>
-          <t>Cat-Skin-&amp;-Coat-Supplement</t>
+      <c r="S75" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>petme2 cat feeder</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>exact</t>
         </is>
       </c>
     </row>
@@ -3520,12 +3541,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>More-Supplement</t>
+          <t>Brand-All</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -3538,7 +3559,7 @@
       </c>
       <c r="T76" t="inlineStr">
         <is>
-          <t>cat skin and coat supplement</t>
+          <t>petme2 cat water fountain</t>
         </is>
       </c>
       <c r="U76" t="inlineStr">
@@ -3555,7 +3576,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Keyword</t>
+          <t>Ad Group</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3565,31 +3586,26 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>More-Supplement</t>
+          <t>Brand-Filters</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Filters - Exact (OUT OF STOCK - paused)</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="S77" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T77" t="inlineStr">
-        <is>
-          <t>cat vitamins for skin and coat</t>
-        </is>
-      </c>
-      <c r="U77" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
+          <t>paused</t>
+        </is>
+      </c>
+      <c r="R77" t="n">
+        <v>0.25</v>
       </c>
     </row>
     <row r="78">
@@ -3600,7 +3616,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Keyword</t>
+          <t>Product Ad</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3610,12 +3626,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>More-Supplement</t>
+          <t>Brand-Filters</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -3623,17 +3639,9 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="S78" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="T78" t="inlineStr">
-        <is>
-          <t>cat shedding supplement</t>
-        </is>
-      </c>
-      <c r="U78" t="inlineStr">
-        <is>
-          <t>exact</t>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>2L-Filter</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3653,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Ad Group</t>
+          <t>Product Ad</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3655,17 +3663,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>More-FeederWaterer</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>Feeder + Waterer - Exact (out of stock)</t>
+          <t>Brand-Filters</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -3673,8 +3676,10 @@
           <t>enabled</t>
         </is>
       </c>
-      <c r="R79" t="n">
-        <v>0.4</v>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>2.2Ltr-Filter-Transparent</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -3695,12 +3700,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>More-FeederWaterer</t>
+          <t>Brand-Filters</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -3710,7 +3715,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>2in1_FEEDER</t>
+          <t>2.2L-Filter</t>
         </is>
       </c>
     </row>
@@ -3732,12 +3737,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>PETME2-SP-AllProducts</t>
+          <t>PETME2-SP-Brand</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>More-FeederWaterer</t>
+          <t>Brand-Filters</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -3747,7 +3752,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>FEEDER_X_WATERER</t>
+          <t>3.2L-Stainless-Steel-Filter</t>
         </is>
       </c>
     </row>
@@ -3759,38 +3764,120 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>Product Ad</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>PETME2-SP-Brand</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Brand-Filters</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>2.2Litre-Filter-Transparent</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Sponsored Products</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
           <t>Keyword</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Create</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>PETME2-SP-AllProducts</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>More-FeederWaterer</t>
-        </is>
-      </c>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="S82" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="T82" t="inlineStr">
-        <is>
-          <t>automatic cat feeder and water dispenser</t>
-        </is>
-      </c>
-      <c r="U82" t="inlineStr">
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>PETME2-SP-Brand</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Brand-Filters</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="S83" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>petme2 filter</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Sponsored Products</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>PETME2-SP-Brand</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Brand-Filters</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="S84" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>petme2 fountain filter</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
         <is>
           <t>exact</t>
         </is>

</xml_diff>

<commit_message>
PETME2: owner product costs, real FBA fees, break-even per product; lower bids on low-margin products
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HHS1qB7cDk7kf96VcdcLix
</commit_message>
<xml_diff>
--- a/petme2-ads-agent/outbox/2026-10-04/bulk-upload-2-new-campaigns.xlsx
+++ b/petme2-ads-agent/outbox/2026-10-04/bulk-upload-2-new-campaigns.xlsx
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -936,7 +936,7 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="S34" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="S36" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
         </is>
       </c>
       <c r="S38" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="S44" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="S45" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="T45" t="inlineStr">
         <is>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="S46" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="T46" t="inlineStr">
         <is>

</xml_diff>